<commit_message>
9/29 neat-freak 同步：台账补 9/26/9/29 至 15 行、新增 HANDOFF.md、作品集/README/CLAUDE.md 对齐、清理调试文件
</commit_message>
<xml_diff>
--- a/demos/作品集总览/AI小工具Demo台账.xlsx
+++ b/demos/作品集总览/AI小工具Demo台账.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI 小工具 Demo 台账（9/14 – 9/25）</t>
+          <t>AI 小工具 Demo 台账（9/14 – 9/29）</t>
         </is>
       </c>
     </row>
@@ -1040,8 +1040,50 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" t="n">
-        <v>12</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>网站数据自动采集器</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>maxun（GitHub）</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4星</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>网页工具</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>配置网址和字段→定时采集→自动对比变化（价格涨跌/新增/下架）→告警→导出CSV</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>已交付</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://aka.doubaocdn.com/s/jdmT6UyrBY</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1135,16 +1177,62 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>说明：共 14 个已交付 demo；9/22 因当日无资讯入库未产出；来源均为「AI工具资讯日报」飞书多维表格，点击链接可直接打开运行。</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AI目标驱动工作流执行器</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Beam AI（Product Hunt）</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>4星</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>网页工具</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>自然语言目标→AI拆解步骤链→调用虚拟工具逐步执行→产出交付物</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>已交付</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://github.com/zhonghugo/Hugo-AI-Tools-Demos/blob/main/demos/2026-09-29_AI目标驱动工作流工具/AI目标驱动工作流执行器.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>说明：共 15 个已交付 demo；9/22 因当日无资讯入库未产出；来源均为「AI工具资讯日报」飞书多维表格，点击链接可直接打开运行。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A14:I14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>

</xml_diff>

<commit_message>
10/28 LLM API成本监控面板 demo
</commit_message>
<xml_diff>
--- a/demos/作品集总览/AI小工具Demo台账.xlsx
+++ b/demos/作品集总览/AI小工具Demo台账.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2490,9 +2490,54 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>说明：共 43 个已交付 demo；9/22 因当日无资讯入库未产出；来源均为「AI工具资讯日报」飞书多维表格，点击链接可直接打开运行。</t>
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>LLM API成本监控面板</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FreeLLMAPI 34家免费provider聚合+智能路由+故障转移</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>4星</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>网页工具</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>参考 FreeLLMAPI「34家免费provider聚合+智能路由+故障转移」（41K stars，自托管LLM路由，每月74亿免费token）：①统一端点——所有 AI 应用（客服机器人/文档处理/数据分析/RPA 智能环节）只配一个 OpenAI 兼容端点，路由与故障转移由网关完成、应用零改动；②Provider 路由总览——8 家 provider（OpenAI/DeepSeek/Gemini/通义/Kimi/Claude/智谱/文心）单价、延迟、免费配额、可用状态可视化；③智能路由——按策略（最低单价/最低延迟/轮询均衡）自动选 Provider，测试请求日志记录每次决策理由；④故障转移——Provider 故障自动绕行切换、请求 0 失败，支持手动模拟故障与一键恢复；⑤成本监控——近 12 天 token 用量趋势图（SVG 柱状）、按 Provider 配额分布、月度成本与预算实时比对；⑥配额预算——74 亿免费 token 配额进度条（占用&gt;80% 预警、&gt;95% 强制降级），月度预算上限+超限告警；把公司 AI 应用 API 成本管起来</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>已交付</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://github.com/zhonghugo/Hugo-AI-Tools-Demos/blob/main/demos/2026-10-28_LLM%20API%E6%88%90%E6%9C%AC%E7%9B%91%E6%8E%A7%E9%9D%A2%E6%9D%BF/LLM%20API%E6%88%90%E6%9C%AC%E7%9B%91%E6%8E%A7%E9%9D%A2%E6%9D%BF.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>说明：共 44 个已交付 demo；9/22 因当日无资讯入库未产出；来源均为「AI工具资讯日报」飞书多维表格，点击链接可直接打开运行。</t>
         </is>
       </c>
     </row>

</xml_diff>